<commit_message>
missing meteo column for postprocessing
</commit_message>
<xml_diff>
--- a/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
+++ b/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="581">
   <si>
     <t xml:space="preserve">Input</t>
   </si>
@@ -1626,6 +1626,9 @@
   </si>
   <si>
     <t xml:space="preserve">Conductance parameter </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;</t>
   </si>
   <si>
     <t xml:space="preserve">water_moisture_patch</t>
@@ -10740,8 +10743,8 @@
         <v>1.2E-005</v>
       </c>
       <c r="K226" s="10" t="n">
-        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 100</f>
-        <v>0.0012</v>
+        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 10</f>
+        <v>0.00012</v>
       </c>
       <c r="L226" s="10" t="n">
         <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2</f>
@@ -10785,7 +10788,7 @@
         <v>35</v>
       </c>
       <c r="K227" s="10" t="s">
-        <v>35</v>
+        <v>535</v>
       </c>
       <c r="L227" s="10" t="s">
         <v>35</v>
@@ -10793,7 +10796,7 @@
     </row>
     <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A228" s="4" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B228" s="8" t="s">
         <v>32</v>
@@ -10805,7 +10808,7 @@
         <v>14</v>
       </c>
       <c r="E228" s="59" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F228" s="59" t="s">
         <v>496</v>
@@ -10851,7 +10854,7 @@
     </row>
     <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="4" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B229" s="8" t="s">
         <v>32</v>
@@ -10863,7 +10866,7 @@
         <v>488</v>
       </c>
       <c r="E229" s="59" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F229" s="59" t="s">
         <v>499</v>
@@ -10909,7 +10912,7 @@
     </row>
     <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="4" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B230" s="8" t="s">
         <v>32</v>
@@ -10921,7 +10924,7 @@
         <v>488</v>
       </c>
       <c r="E230" s="59" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="F230" s="59" t="s">
         <v>499</v>
@@ -10972,7 +10975,7 @@
     </row>
     <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="4" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B231" s="8" t="s">
         <v>32</v>
@@ -10984,7 +10987,7 @@
         <v>488</v>
       </c>
       <c r="E231" s="59" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F231" s="59" t="s">
         <v>499</v>
@@ -11030,7 +11033,7 @@
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A232" s="4" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B232" s="8" t="s">
         <v>32</v>
@@ -11042,10 +11045,10 @@
         <v>14</v>
       </c>
       <c r="E232" s="59" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="F232" s="59" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="G232" s="10" t="n">
         <v>1E-005</v>
@@ -11092,7 +11095,7 @@
     </row>
     <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A233" s="4" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B233" s="8" t="s">
         <v>32</v>
@@ -11104,7 +11107,7 @@
         <v>14</v>
       </c>
       <c r="E233" s="59" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F233" s="59" t="s">
         <v>499</v>
@@ -11154,7 +11157,7 @@
     </row>
     <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="4" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B234" s="8" t="s">
         <v>32</v>
@@ -11198,7 +11201,7 @@
     </row>
     <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="4" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B235" s="8" t="s">
         <v>32</v>
@@ -11242,7 +11245,7 @@
     </row>
     <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="1" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B236" s="8" t="s">
         <v>32</v>
@@ -11254,7 +11257,7 @@
         <v>14</v>
       </c>
       <c r="E236" s="54" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F236" s="54" t="s">
         <v>264</v>
@@ -11285,7 +11288,7 @@
     </row>
     <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="42" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B237" s="8" t="s">
         <v>32</v>
@@ -11297,10 +11300,10 @@
         <v>14</v>
       </c>
       <c r="E237" s="43" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F237" s="43" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G237" s="10" t="n">
         <v>1E-009</v>
@@ -11324,7 +11327,7 @@
     </row>
     <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A238" s="42" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B238" s="8" t="s">
         <v>32</v>
@@ -11336,10 +11339,10 @@
         <v>14</v>
       </c>
       <c r="E238" s="43" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="F238" s="43" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="G238" s="10" t="n">
         <v>1E-009</v>
@@ -11363,7 +11366,7 @@
     </row>
     <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A239" s="4" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B239" s="8" t="s">
         <v>32</v>
@@ -11375,10 +11378,10 @@
         <v>14</v>
       </c>
       <c r="E239" s="59" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F239" s="59" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="G239" s="59" t="n">
         <v>0.1</v>
@@ -21290,18 +21293,18 @@
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>31</v>
@@ -21364,7 +21367,7 @@
         <v>159</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C7" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A7,$B$2:$B$170,1,FALSE())),A7,"")</f>
@@ -21601,7 +21604,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>105</v>
@@ -21613,7 +21616,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>107</v>
@@ -21625,7 +21628,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>110</v>
@@ -21637,7 +21640,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>112</v>
@@ -21793,7 +21796,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>161</v>
@@ -21805,7 +21808,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>163</v>
@@ -21817,7 +21820,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>168</v>
@@ -21829,7 +21832,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>173</v>
@@ -21853,7 +21856,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>181</v>
@@ -21865,7 +21868,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>184</v>
@@ -21877,7 +21880,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="2" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="B50" s="2" t="s">
         <v>175</v>
@@ -22084,7 +22087,7 @@
         <v>354</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C67" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A67,$B$2:$B$170,1,FALSE())),A67,"")</f>
@@ -22096,7 +22099,7 @@
         <v>357</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="C68" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A68,$B$2:$B$170,1,FALSE())),A68,"")</f>
@@ -22108,7 +22111,7 @@
         <v>359</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="C69" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A69,$B$2:$B$170,1,FALSE())),A69,"")</f>
@@ -22120,7 +22123,7 @@
         <v>361</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="C70" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A70,$B$2:$B$170,1,FALSE())),A70,"")</f>
@@ -22225,7 +22228,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B79" s="2" t="s">
         <v>318</v>
@@ -22636,7 +22639,7 @@
         <v>461</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="C113" s="2" t="str">
         <f aca="false">IF(ISNA(VLOOKUP(A113,$B$2:$B$170,1,FALSE())),A113,"")</f>
@@ -22801,7 +22804,7 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="2" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>419</v>
@@ -22813,7 +22816,7 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="2" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>421</v>
@@ -22825,7 +22828,7 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="2" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>423</v>
@@ -22837,7 +22840,7 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="2" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>425</v>
@@ -22897,7 +22900,7 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="2" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>436</v>

</xml_diff>

<commit_message>
Shoot allocation to roots sensitive to nitrate export
</commit_message>
<xml_diff>
--- a/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
+++ b/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">WB_defense1</t>
   </si>
   <si>
-    <t xml:space="preserve">GB_CNW_1</t>
+    <t xml:space="preserve">GB_1.0</t>
   </si>
   <si>
     <t xml:space="preserve">GB_CN_1</t>
@@ -11346,8 +11346,8 @@
         <v>6E-007</v>
       </c>
       <c r="K224" s="10" t="n">
-        <f aca="false">0.00001 / 10 / 5 / 10 * 6 * 5</f>
-        <v>6E-007</v>
+        <f aca="false">0.00001 / 10 / 5 / 10 * 6 * 100</f>
+        <v>1.2E-005</v>
       </c>
       <c r="L224" s="10" t="n">
         <f aca="false">0.00001 / 10 / 5 / 10 * 6 * 5</f>
@@ -11446,8 +11446,8 @@
         <v>1.2E-005</v>
       </c>
       <c r="K226" s="10" t="n">
-        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 10</f>
-        <v>0.00012</v>
+        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2</f>
+        <v>1.2E-005</v>
       </c>
       <c r="L226" s="10" t="n">
         <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 10</f>

</xml_diff>

<commit_message>
changed shoot-root water coupling boundary condition and associated shoot psi_ref and GAMMA parameters + missing stomatal model passing
</commit_message>
<xml_diff>
--- a/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
+++ b/simulations/hydro/inputs/Scenarios_26-08-04.xlsx
@@ -11682,8 +11682,8 @@
         <v>0.00012</v>
       </c>
       <c r="M226" s="10" t="n">
-        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2</f>
-        <v>1.2E-005</v>
+        <f aca="false">0.00001 /5 /2/4 * 4 * 0.6 * 10*2 * 10</f>
+        <v>0.00012</v>
       </c>
       <c r="N226" s="11"/>
       <c r="O226" s="59"/>
@@ -17311,7 +17311,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I226:L226">
+  <conditionalFormatting sqref="I226:M226">
     <cfRule type="colorScale" priority="449">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -27047,7 +27047,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M226">
+  <conditionalFormatting sqref="M228:M231">
     <cfRule type="colorScale" priority="1334">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -27069,7 +27069,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M228:M231">
+  <conditionalFormatting sqref="M234:M235">
     <cfRule type="colorScale" priority="1336">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -27091,7 +27091,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M234:M235">
+  <conditionalFormatting sqref="M236">
     <cfRule type="colorScale" priority="1338">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -27113,7 +27113,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M236">
+  <conditionalFormatting sqref="M238">
     <cfRule type="colorScale" priority="1340">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -27125,28 +27125,6 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="1341">
-      <colorScale>
-        <cfvo type="min" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max" val="0"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M238">
-    <cfRule type="colorScale" priority="1342">
-      <colorScale>
-        <cfvo type="min" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max" val="0"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="1343">
       <colorScale>
         <cfvo type="min" val="0"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>